<commit_message>
test: record sprint 1 execution results
</commit_message>
<xml_diff>
--- a/outputs/sprint-1-testing/plan-pruebas-sprint-1.xlsx
+++ b/outputs/sprint-1-testing/plan-pruebas-sprint-1.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de pruebas" sheetId="1" r:id="R5e0f45211e0c4de2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="R106f863d68da4c8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="3" r:id="R58e1a2cf81a34191"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de pruebas" sheetId="1" r:id="R58956fb475cc42c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="Re8b4071f15be4606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="3" r:id="R5846121926264619"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,6 +15,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:numFmts count="1">
+    <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
+  </x:numFmts>
   <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
@@ -168,7 +171,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="62">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -306,6 +309,15 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -772,9 +784,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H2" s="46" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I2" s="40" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I2" s="59" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J2" s="23" t="str"/>
     </x:row>
     <x:row r="3" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -800,9 +814,11 @@
         <x:v>Regression</x:v>
       </x:c>
       <x:c r="H3" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I3" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I3" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J3" s="25" t="str"/>
     </x:row>
     <x:row r="4" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -830,7 +846,7 @@
       <x:c r="H4" s="47" t="str">
         <x:v>Pendiente</x:v>
       </x:c>
-      <x:c r="I4" s="41" t="str"/>
+      <x:c r="I4" s="60"/>
       <x:c r="J4" s="25" t="str"/>
     </x:row>
     <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -856,9 +872,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H5" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I5" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I5" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J5" s="25" t="str"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
@@ -884,9 +902,11 @@
         <x:v>Regression</x:v>
       </x:c>
       <x:c r="H6" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I6" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I6" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J6" s="25" t="str"/>
     </x:row>
     <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -912,9 +932,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H7" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I7" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I7" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J7" s="25" t="str"/>
     </x:row>
     <x:row r="8" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -940,9 +962,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H8" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I8" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I8" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J8" s="25" t="str"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
@@ -968,9 +992,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H9" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I9" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I9" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J9" s="25" t="str"/>
     </x:row>
     <x:row r="10" ht="26.399999618530273" hidden="0" customHeight="1">
@@ -996,9 +1022,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H10" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I10" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I10" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J10" s="25" t="str"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
@@ -1024,9 +1052,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H11" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I11" s="41" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I11" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J11" s="25" t="str"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -1052,9 +1082,11 @@
         <x:v>Regression</x:v>
       </x:c>
       <x:c r="H12" s="48" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I12" s="42" t="str"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J12" s="27" t="str"/>
     </x:row>
   </x:sheetData>
@@ -1108,24 +1140,14 @@
       </x:c>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="58" t="str">
-        <x:v>DEF-01</x:v>
-      </x:c>
-      <x:c r="B2" s="56" t="str">
-        <x:v>Completar al detectar un defecto</x:v>
-      </x:c>
-      <x:c r="C2" s="56" t="str">
-        <x:v>Media</x:v>
-      </x:c>
-      <x:c r="D2" s="56" t="str">
-        <x:v>localhost:5173</x:v>
-      </x:c>
-      <x:c r="E2" s="56" t="str"/>
-      <x:c r="F2" s="56" t="str"/>
-      <x:c r="G2" s="56" t="str"/>
-      <x:c r="H2" s="57" t="str">
-        <x:v>Abierto</x:v>
-      </x:c>
+      <x:c r="A2" s="58"/>
+      <x:c r="B2" s="56"/>
+      <x:c r="C2" s="56"/>
+      <x:c r="D2" s="56"/>
+      <x:c r="E2" s="56"/>
+      <x:c r="F2" s="56"/>
+      <x:c r="G2" s="56"/>
+      <x:c r="H2" s="57"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="2">

</xml_diff>

<commit_message>
test: complete sprint 1 manual test execution
</commit_message>
<xml_diff>
--- a/outputs/sprint-1-testing/plan-pruebas-sprint-1.xlsx
+++ b/outputs/sprint-1-testing/plan-pruebas-sprint-1.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de pruebas" sheetId="1" r:id="R58956fb475cc42c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="Re8b4071f15be4606"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="3" r:id="R5846121926264619"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plan de pruebas" sheetId="1" r:id="R4b02c232a5a346f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Casos de prueba" sheetId="2" r:id="Rdae8d87bc5a548a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Defectos" sheetId="3" r:id="Re5bd5a692f05468f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -844,9 +844,11 @@
         <x:v>Smoke</x:v>
       </x:c>
       <x:c r="H4" s="47" t="str">
-        <x:v>Pendiente</x:v>
-      </x:c>
-      <x:c r="I4" s="60"/>
+        <x:v>Aprobado</x:v>
+      </x:c>
+      <x:c r="I4" s="60" t="n">
+        <x:v>46278</x:v>
+      </x:c>
       <x:c r="J4" s="25" t="str"/>
     </x:row>
     <x:row r="5" ht="26.399999618530273" hidden="0" customHeight="1">

</xml_diff>